<commit_message>
TechStack: add Mac-Local Feasibility sheet (full skills matrix)
- map the 43-area skills matrix to Mac-local feasibility on synthetic data:
  28 fully local, 8 local-capable, 2 cloud-only (Azure), 5 optional/soft
- reframe DL rows to Mac (MPS) / Cloud — small synthetic data trains on M3 Pro
- Overview: local-first philosophy; note cloud-only = Azure (sub: MLflow),
  MATLAB skipped; Spark local mode, single-node k8s (kind/minikube), CI via act
- note for Task 1: whole pipeline is Mac-local
</commit_message>
<xml_diff>
--- a/docs/TechStack.xlsx
+++ b/docs/TechStack.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tech Stack" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Mac-Local Feasibility" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +37,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00004B93"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +67,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBF3E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -108,6 +123,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -216,6 +240,36 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="495300" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -534,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -593,43 +647,55 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Light core runs on the Mac; heavy deep-learning + MLOps run on non-Apple cloud GPU. Deps are staged by task, pinned, and reproducible.</t>
+          <t>Because the data is SYNTHETIC (small), the whole stack runs LOCAL-FIRST on the Mac — including deep learning via PyTorch MPS (Metal). Cloud is optional, only for scale or the real public deployment.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Guardrails</t>
+          <t>Mac-local (Task 1)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>No Apple ecosystem; personal GitHub; Mac never runs heavy training.</t>
+          <t>Almost everything runs completely on the Mac. Cloud-only = Azure ML / Azure Cloud (substitute with MLflow + non-Apple cloud for real deploy); MATLAB skipped (licensed). See the 'Mac-Local Feasibility' sheet.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Status legend</t>
+          <t>Guardrails</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Installed / In use / Done = available now (green). Planned = introduced at a later task (amber).</t>
+          <t>No Apple ecosystem; personal GitHub. Mac stays comfortable because synthetic data is small; a --sample flag + optional cloud cover any scale-up.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>Status legend</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Installed / In use / Done = available now (green). Planned = introduced at a later task (amber).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>See also</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Task0_Summary.xlsx (scope, brands, channels, architecture) and README.md (roadmap).</t>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Mac-Local Feasibility sheet (this file); Task0_Summary.xlsx (scope/brands/channels/architecture); README.md (roadmap).</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1577,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Cloud (GPU)</t>
+          <t>Mac (MPS) / Cloud</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1605,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Cloud (GPU)</t>
+          <t>Mac (MPS) / Cloud</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1633,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Cloud (GPU)</t>
+          <t>Mac (MPS) / Cloud</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1661,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Cloud (GPU)</t>
+          <t>Mac (MPS) / Cloud</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1721,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Cloud (GPU)</t>
+          <t>Mac / Cloud</t>
         </is>
       </c>
     </row>
@@ -2198,4 +2264,1233 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Mac-Local Feasibility — full skills matrix on synthetic data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Area / Stack</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Technologies</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Mac-local?</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>How on the Mac (local tool / substitute)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Programming</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Python 3.12 venv</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Task 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Additional languages</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>R, Scala, MATLAB</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Optional/soft</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>R via brew; Scala on the JVM (with Spark); MATLAB is licensed -&gt; skip</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Python ML production</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>scikit-learn, ML pipelines</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>sklearn Pipelines on synthetic data</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Task 4-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Data science</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>ML, statistics, business modeling</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>numpy / scipy / sklearn + notebooks</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Python engineering</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>OOP, modular programming</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>src/ package layout (in progress)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Task 0+</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>pytest / unit testing</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>pytest wired via pre-commit</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Task 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Code quality</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>PEP8, Black</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>ruff + black + pre-commit</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Task 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Scientific Python</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>pandas, NumPy, SciPy, scikit-learn, Matplotlib</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>core deps already installed</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Task 1-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Classical time series</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ARIMA, SARIMA, SARIMAX</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>statsmodels, pmdarima</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Statistical forecasting</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Exponential Smoothing, ETS, state-space</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>statsmodels</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Prophet</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Prophet</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>pip install prophet (cmdstanpy) — CPU</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Multivariate time series</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>statsmodels VAR</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>ML forecasting</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>XGBoost, LightGBM</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>CPU training on synthetic data</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Deep learning</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>LSTM, GRU (PyTorch)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>PyTorch MPS (Metal) — small synthetic data trains on M3 Pro</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Task 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Transformer forecasting</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>TFT / Transformer TS</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>PyTorch MPS; small models; cloud only if scaling up</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Task 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Time-series features</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>lags, rolling stats, calendar, exogenous</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>pandas feature pipeline</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Task 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Trend &amp; seasonality</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>decomposition, seasonal patterns</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>statsmodels STL</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Task 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Anomaly detection</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>TS anomaly / outlier detection</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>statsmodels / sklearn / alibi-detect (CPU)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Task 2/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Backtesting</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>rolling / expanding window</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>custom harness + sklearn TimeSeriesSplit</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Forecast metrics</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>MAE, RMSE, MAPE, sMAPE, WAPE, WRMSSE</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>metrics module</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Task 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Bayesian modeling</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Bayesian inference, probabilistic</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>PyMC / NumPyro — CPU sampling on small data</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Task 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Probabilistic forecasting</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>prediction distributions / uncertainty</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>quantile loss, DeepAR (small), PyMC</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Task 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Big data</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Apache Spark</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>PySpark local[*] mode + Java (brew) — single machine</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Task 3/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Relational databases</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>SQL, RDBMS</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>DuckDB + SQLite (serverless); Postgres via Docker</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Task 1/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>NoSQL</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>NoSQL databases</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>MongoDB via Docker (optional)</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Azure ML</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Azure Machine Learning</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Cloud-only</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Substitute locally with MLflow (tracking + registry)</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Task 11 (sub)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Azure cloud</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Azure services</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Cloud-only</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Emulate locally; real deploy -&gt; non-Apple cloud (Render / Cloud Run)</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Task 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>REST APIs</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>FastAPI, Flask</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>uvicorn on localhost</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Task 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Microservices</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>REST services, integration</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>docker-compose multi-service</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Task 14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Frontend collaboration</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>React, Angular</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Node + Vite React demo (HTML mockup already built)</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Task 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Containers</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Docker</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Docker Desktop (Apple Silicon)</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Task 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Orchestration</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Kubernetes</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>kind / minikube / k3d single-node on the Mac</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Task 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Version control</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Git</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>git + GitHub</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Task 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>CI/CD</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>CI/CD pipelines</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>pre-commit now; GitHub Actions emulated locally with `act`</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Task 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>DevOps / MLOps</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Docker, Kubernetes, CI/CD, cloud</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>docker + local k8s + MLflow + act</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Task 12-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>logging, monitoring, alerting</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>structured logging; Prometheus + Grafana via docker-compose; Evidently</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Task 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>secure production practices</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>FastAPI JWT/OAuth2, .env secrets, RBAC</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Task 14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>End-to-end data products</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Data -&gt; ML -&gt; API -&gt; app -&gt; monitoring</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Fully local</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>the whole pipeline runs on the Mac</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Production deployment</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>model serving, deploy, monitor</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Local-capable</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>local docker/k8s emulation; real endpoint -&gt; non-Apple cloud</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Task 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Product thinking</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>architecture + business integration</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Optional/soft</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>docs, Architecture sheet, README</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Professional skills</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>communication, service orientation</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Optional/soft</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>demonstrated via docs / deck</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Teamwork</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>collaboration + autonomous delivery</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Optional/soft</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>git workflow, branches, PRs</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>fluent English</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Optional/soft</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>docs, deck, code comments</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="58" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Verdict: with synthetic data, 28/43 areas run FULLY on the Mac and most of the rest are local-capable (Spark local mode, single-node Kubernetes via kind/minikube, CI via `act`, DL via PyTorch MPS). Only Azure ML / Azure Cloud are cloud-only (substitute: MLflow locally + a non-Apple cloud for the one real-deployment task). MATLAB is skipped (licensed).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A46:E46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>